<commit_message>
Ajout des défis AWS EC2 dans le fichier de pannes IT
</commit_message>
<xml_diff>
--- a/incident-log-pannes-IT.xlsx
+++ b/incident-log-pannes-IT.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\mes-pannes-IT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B74A9F83-7A36-49BF-8D50-2110054CF30E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A51DEFA5-E1F3-48B6-9456-930C1A16458B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
   <si>
     <t>Problème n°</t>
   </si>
@@ -127,6 +127,109 @@
 Erreur observée :
 Permission denied (publickey)
 fatal: Could not read from remote repository</t>
+  </si>
+  <si>
+    <t>Ex.3</t>
+  </si>
+  <si>
+    <t>exemple 3</t>
+  </si>
+  <si>
+    <t>AWS / Cloud Infrastructure</t>
+  </si>
+  <si>
+    <t>Impossible de se connecter à 
+l’instance EC2 Misconfigured
+ Web Server via EC2
+ Instance Connect.</t>
+  </si>
+  <si>
+    <t>La connexion EC2 Instance Connec
+t échoue. Le terminal ne s’ouvre 
+pas ou affiche une erreur de
+ connexion SSH.</t>
+  </si>
+  <si>
+    <t>Le Security Group associé
+ à l’instance EC2
+ ne permettait pas le trafic
+ entrant sur le port 22 (SSH).
+ Sans cette règle,
+ la connexion SSH est bloquée.</t>
+  </si>
+  <si>
+    <t>Vérifier le Security Group
+ de l’instance. Modifier les
+ Inbound Rules. Ajouter une
+ règle autorisant SSH (port 22
+) depuis Internet. Réessayer
+ la connexion via EC2
+ Instance Connect.</t>
+  </si>
+  <si>
+    <t>.AWS Management Console
+. EC2 Instance Connec
+.Security Groups</t>
+  </si>
+  <si>
+    <t>Ce problème est fréquent
+ lors de la configuration
+ initiale d’une instance
+ EC2 si les règles de sécurité
+ ne sont pas correctement définies.</t>
+  </si>
+  <si>
+    <t>Ex.4</t>
+  </si>
+  <si>
+    <t>exemple 4</t>
+  </si>
+  <si>
+    <t>AWS / Web Server 
+Configuration</t>
+  </si>
+  <si>
+    <t>Le serveur web installé 
+sur l’instance EC2 n’était
+ pas accessible via
+ son Public IPv4 DNS</t>
+  </si>
+  <si>
+    <t>La page web ne s’affiche pas dans
+ le navigateur après avoir saisi
+ le Public DNS. Le navigateur
+ affiche une erreur de connexion.</t>
+  </si>
+  <si>
+    <t>Le service Apache (httpd) 
+n’était pas installé ou démarré
+ sur l’instance EC2 et le port
+ 80 (HTTP) n’était pas
+ autorisé dans le Security Group.</t>
+  </si>
+  <si>
+    <t>Se connecter à l’instance EC2
+. Installer Apache avec sudo
+ yum install httpd -y. Démarrer
+ le service avec sudo systemctl
+ start httpd. Activer le service
+ avec sudo systemctl enable 
+httpd. Ajouter une règle
+ HTTP (port 80) dans 
+le Security Group.</t>
+  </si>
+  <si>
+    <t>.EC2 Instance Connect
+. Linux Terminal
+. Apache HTTP Server
+. AWS Security Groups</t>
+  </si>
+  <si>
+    <t>Vérifier toujours les services 
+actifs sur l’instance et les 
+règles réseau lorsque
+ l’accès à une application
+ web échoue.</t>
   </si>
 </sst>
 </file>
@@ -211,10 +314,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -230,40 +331,48 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -566,7 +675,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -578,288 +687,545 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="14" t="s">
+      <c r="I1" s="11" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="C2" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="D2" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="E2" s="11" t="s">
+      <c r="E2" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="F2" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="13" t="s">
+      <c r="G2" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="H2" s="17"/>
-      <c r="I2" s="14"/>
+      <c r="H2" s="6"/>
+      <c r="I2" s="11"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A3" s="2"/>
-      <c r="B3" s="6"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="11"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
-      <c r="H3" s="19" t="s">
+      <c r="A3" s="21"/>
+      <c r="B3" s="4"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="15"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="I3" s="14"/>
+      <c r="I3" s="11"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A4" s="2"/>
-      <c r="B4" s="6"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="13"/>
-      <c r="G4" s="13"/>
+      <c r="A4" s="21"/>
+      <c r="B4" s="4"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="15"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
       <c r="H4" s="18"/>
-      <c r="I4" s="14"/>
+      <c r="I4" s="11"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A5" s="2"/>
-      <c r="B5" s="16"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="13"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="13"/>
-      <c r="G5" s="13"/>
+      <c r="A5" s="21"/>
+      <c r="B5" s="19"/>
+      <c r="C5" s="20"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
       <c r="H5" s="18"/>
-      <c r="I5" s="14"/>
+      <c r="I5" s="11"/>
     </row>
     <row r="6" spans="1:9" ht="29" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="2"/>
-      <c r="B6" s="16"/>
-      <c r="C6" s="10"/>
-      <c r="D6" s="13"/>
-      <c r="E6" s="11"/>
-      <c r="F6" s="13"/>
-      <c r="G6" s="13"/>
+      <c r="A6" s="21"/>
+      <c r="B6" s="19"/>
+      <c r="C6" s="20"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="15"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="9"/>
       <c r="H6" s="18"/>
-      <c r="I6" s="14"/>
+      <c r="I6" s="11"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A7" s="2"/>
-      <c r="B7" s="16"/>
-      <c r="C7" s="10"/>
-      <c r="D7" s="13"/>
-      <c r="E7" s="11"/>
-      <c r="F7" s="13"/>
-      <c r="G7" s="13"/>
+      <c r="A7" s="21"/>
+      <c r="B7" s="19"/>
+      <c r="C7" s="20"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="15"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
       <c r="H7" s="18"/>
-      <c r="I7" s="14"/>
+      <c r="I7" s="11"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A8" s="2"/>
-      <c r="B8" s="16"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="13"/>
-      <c r="E8" s="11"/>
-      <c r="F8" s="13"/>
-      <c r="G8" s="13"/>
+      <c r="A8" s="21"/>
+      <c r="B8" s="19"/>
+      <c r="C8" s="20"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="9"/>
       <c r="H8" s="18"/>
-      <c r="I8" s="14"/>
+      <c r="I8" s="11"/>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A9" s="2"/>
-      <c r="B9" s="16"/>
-      <c r="C9" s="10"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="13"/>
-      <c r="G9" s="13"/>
+      <c r="A9" s="21"/>
+      <c r="B9" s="19"/>
+      <c r="C9" s="20"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="9"/>
       <c r="H9" s="18"/>
-      <c r="I9" s="14"/>
+      <c r="I9" s="11"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A10" s="2"/>
-      <c r="B10" s="16"/>
-      <c r="C10" s="10"/>
-      <c r="D10" s="13"/>
-      <c r="E10" s="11"/>
-      <c r="F10" s="13"/>
-      <c r="G10" s="13"/>
+      <c r="A10" s="21"/>
+      <c r="B10" s="19"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="9"/>
       <c r="H10" s="18"/>
-      <c r="I10" s="14"/>
+      <c r="I10" s="11"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A11" s="15" t="s">
+      <c r="A11" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="16" t="s">
+      <c r="B11" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="C11" s="13" t="s">
+      <c r="C11" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="11" t="s">
+      <c r="D11" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="E11" s="11" t="s">
+      <c r="E11" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="F11" s="12" t="s">
+      <c r="F11" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="G11" s="13" t="s">
+      <c r="G11" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="I11" s="14"/>
+      <c r="I11" s="11"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A12" s="15"/>
-      <c r="B12" s="16"/>
-      <c r="C12" s="8"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="1"/>
-      <c r="G12" s="8"/>
-      <c r="H12" s="11" t="s">
+      <c r="A12" s="12"/>
+      <c r="B12" s="19"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="16"/>
+      <c r="E12" s="16"/>
+      <c r="F12" s="16"/>
+      <c r="G12" s="10"/>
+      <c r="H12" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="I12" s="14" t="s">
+      <c r="I12" s="11" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A13" s="15"/>
-      <c r="B13" s="16"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="9"/>
-      <c r="F13" s="1"/>
-      <c r="G13" s="8"/>
-      <c r="H13" s="9"/>
-      <c r="I13" s="14"/>
+      <c r="A13" s="12"/>
+      <c r="B13" s="19"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="16"/>
+      <c r="F13" s="16"/>
+      <c r="G13" s="10"/>
+      <c r="H13" s="16"/>
+      <c r="I13" s="11"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A14" s="15"/>
-      <c r="B14" s="16"/>
-      <c r="C14" s="8"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="1"/>
-      <c r="G14" s="8"/>
-      <c r="H14" s="9"/>
-      <c r="I14" s="14"/>
+      <c r="A14" s="12"/>
+      <c r="B14" s="19"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="16"/>
+      <c r="E14" s="16"/>
+      <c r="F14" s="16"/>
+      <c r="G14" s="10"/>
+      <c r="H14" s="16"/>
+      <c r="I14" s="11"/>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A15" s="15"/>
-      <c r="B15" s="16"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="9"/>
-      <c r="F15" s="1"/>
-      <c r="G15" s="8"/>
-      <c r="H15" s="9"/>
-      <c r="I15" s="14"/>
+      <c r="A15" s="12"/>
+      <c r="B15" s="19"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="16"/>
+      <c r="F15" s="16"/>
+      <c r="G15" s="10"/>
+      <c r="H15" s="16"/>
+      <c r="I15" s="11"/>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A16" s="15"/>
-      <c r="B16" s="16"/>
-      <c r="C16" s="8"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="9"/>
-      <c r="F16" s="1"/>
-      <c r="G16" s="8"/>
-      <c r="H16" s="9"/>
-      <c r="I16" s="14"/>
+      <c r="A16" s="12"/>
+      <c r="B16" s="19"/>
+      <c r="C16" s="10"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="16"/>
+      <c r="F16" s="16"/>
+      <c r="G16" s="10"/>
+      <c r="H16" s="16"/>
+      <c r="I16" s="11"/>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A17" s="15"/>
-      <c r="B17" s="16"/>
-      <c r="C17" s="8"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="9"/>
-      <c r="F17" s="1"/>
-      <c r="G17" s="8"/>
-      <c r="H17" s="9"/>
-      <c r="I17" s="14"/>
+      <c r="A17" s="12"/>
+      <c r="B17" s="19"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="16"/>
+      <c r="F17" s="16"/>
+      <c r="G17" s="10"/>
+      <c r="H17" s="16"/>
+      <c r="I17" s="11"/>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A18" s="15"/>
-      <c r="B18" s="16"/>
-      <c r="C18" s="8"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="9"/>
-      <c r="F18" s="1"/>
-      <c r="G18" s="8"/>
-      <c r="H18" s="9"/>
-      <c r="I18" s="14"/>
+      <c r="A18" s="12"/>
+      <c r="B18" s="19"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="16"/>
+      <c r="F18" s="16"/>
+      <c r="G18" s="10"/>
+      <c r="H18" s="16"/>
+      <c r="I18" s="11"/>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A19" s="15"/>
-      <c r="B19" s="16"/>
-      <c r="C19" s="8"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="1"/>
-      <c r="G19" s="8"/>
-      <c r="H19" s="9"/>
-      <c r="I19" s="14"/>
+      <c r="A19" s="12"/>
+      <c r="B19" s="19"/>
+      <c r="C19" s="10"/>
+      <c r="D19" s="16"/>
+      <c r="E19" s="16"/>
+      <c r="F19" s="16"/>
+      <c r="G19" s="10"/>
+      <c r="H19" s="16"/>
+      <c r="I19" s="11"/>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A20" s="15"/>
-      <c r="B20" s="16"/>
-      <c r="C20" s="8"/>
-      <c r="D20" s="9"/>
-      <c r="E20" s="9"/>
-      <c r="F20" s="1"/>
-      <c r="G20" s="8"/>
-      <c r="H20" s="9"/>
-      <c r="I20" s="14"/>
+      <c r="A20" s="12"/>
+      <c r="B20" s="19"/>
+      <c r="C20" s="10"/>
+      <c r="D20" s="16"/>
+      <c r="E20" s="16"/>
+      <c r="F20" s="16"/>
+      <c r="G20" s="10"/>
+      <c r="H20" s="16"/>
+      <c r="I20" s="11"/>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A21" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="B21" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="C21" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="F21" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="G21" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="H21" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="I21" s="11" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A22" s="12"/>
+      <c r="B22" s="19"/>
+      <c r="C22" s="10"/>
+      <c r="D22" s="10"/>
+      <c r="E22" s="10"/>
+      <c r="F22" s="10"/>
+      <c r="G22" s="10"/>
+      <c r="H22" s="10"/>
+      <c r="I22" s="11"/>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A23" s="12"/>
+      <c r="B23" s="19"/>
+      <c r="C23" s="10"/>
+      <c r="D23" s="10"/>
+      <c r="E23" s="10"/>
+      <c r="F23" s="10"/>
+      <c r="G23" s="10"/>
+      <c r="H23" s="10"/>
+      <c r="I23" s="11"/>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A24" s="12"/>
+      <c r="B24" s="19"/>
+      <c r="C24" s="10"/>
+      <c r="D24" s="10"/>
+      <c r="E24" s="10"/>
+      <c r="F24" s="10"/>
+      <c r="G24" s="10"/>
+      <c r="H24" s="10"/>
+      <c r="I24" s="11"/>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A25" s="12"/>
+      <c r="B25" s="19"/>
+      <c r="C25" s="10"/>
+      <c r="D25" s="10"/>
+      <c r="E25" s="10"/>
+      <c r="F25" s="10"/>
+      <c r="G25" s="10"/>
+      <c r="H25" s="10"/>
+      <c r="I25" s="11"/>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A26" s="12"/>
+      <c r="B26" s="19"/>
+      <c r="C26" s="10"/>
+      <c r="D26" s="10"/>
+      <c r="E26" s="10"/>
+      <c r="F26" s="10"/>
+      <c r="G26" s="10"/>
+      <c r="H26" s="10"/>
+      <c r="I26" s="11"/>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A27" s="12"/>
+      <c r="B27" s="19"/>
+      <c r="C27" s="10"/>
+      <c r="D27" s="10"/>
+      <c r="E27" s="10"/>
+      <c r="F27" s="10"/>
+      <c r="G27" s="10"/>
+      <c r="H27" s="10"/>
+      <c r="I27" s="11"/>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A28" s="12"/>
+      <c r="B28" s="19"/>
+      <c r="C28" s="10"/>
+      <c r="D28" s="10"/>
+      <c r="E28" s="10"/>
+      <c r="F28" s="10"/>
+      <c r="G28" s="10"/>
+      <c r="H28" s="10"/>
+      <c r="I28" s="11"/>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A29" s="12"/>
+      <c r="B29" s="19"/>
+      <c r="C29" s="10"/>
+      <c r="D29" s="10"/>
+      <c r="E29" s="10"/>
+      <c r="F29" s="10"/>
+      <c r="G29" s="10"/>
+      <c r="H29" s="10"/>
+      <c r="I29" s="11"/>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A30" s="12"/>
+      <c r="B30" s="19"/>
+      <c r="C30" s="10"/>
+      <c r="D30" s="10"/>
+      <c r="E30" s="10"/>
+      <c r="F30" s="10"/>
+      <c r="G30" s="10"/>
+      <c r="H30" s="10"/>
+      <c r="I30" s="11"/>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A31" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="B31" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="C31" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="D31" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="E31" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="F31" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="G31" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="H31" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="I31" s="11" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A32" s="12"/>
+      <c r="B32" s="14"/>
+      <c r="C32" s="10"/>
+      <c r="D32" s="10"/>
+      <c r="E32" s="10"/>
+      <c r="F32" s="8"/>
+      <c r="G32" s="10"/>
+      <c r="H32" s="10"/>
+      <c r="I32" s="11"/>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A33" s="12"/>
+      <c r="B33" s="14"/>
+      <c r="C33" s="10"/>
+      <c r="D33" s="10"/>
+      <c r="E33" s="10"/>
+      <c r="F33" s="8"/>
+      <c r="G33" s="10"/>
+      <c r="H33" s="10"/>
+      <c r="I33" s="11"/>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A34" s="12"/>
+      <c r="B34" s="14"/>
+      <c r="C34" s="10"/>
+      <c r="D34" s="10"/>
+      <c r="E34" s="10"/>
+      <c r="F34" s="8"/>
+      <c r="G34" s="10"/>
+      <c r="H34" s="10"/>
+      <c r="I34" s="11"/>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A35" s="12"/>
+      <c r="B35" s="14"/>
+      <c r="C35" s="10"/>
+      <c r="D35" s="10"/>
+      <c r="E35" s="10"/>
+      <c r="F35" s="8"/>
+      <c r="G35" s="10"/>
+      <c r="H35" s="10"/>
+      <c r="I35" s="11"/>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A36" s="12"/>
+      <c r="B36" s="14"/>
+      <c r="C36" s="10"/>
+      <c r="D36" s="10"/>
+      <c r="E36" s="10"/>
+      <c r="F36" s="8"/>
+      <c r="G36" s="10"/>
+      <c r="H36" s="10"/>
+      <c r="I36" s="11"/>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A37" s="12"/>
+      <c r="B37" s="14"/>
+      <c r="C37" s="10"/>
+      <c r="D37" s="10"/>
+      <c r="E37" s="10"/>
+      <c r="F37" s="8"/>
+      <c r="G37" s="10"/>
+      <c r="H37" s="10"/>
+      <c r="I37" s="11"/>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A38" s="12"/>
+      <c r="B38" s="14"/>
+      <c r="C38" s="10"/>
+      <c r="D38" s="10"/>
+      <c r="E38" s="10"/>
+      <c r="F38" s="8"/>
+      <c r="G38" s="10"/>
+      <c r="H38" s="10"/>
+      <c r="I38" s="11"/>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A39" s="12"/>
+      <c r="B39" s="14"/>
+      <c r="C39" s="10"/>
+      <c r="D39" s="10"/>
+      <c r="E39" s="10"/>
+      <c r="F39" s="8"/>
+      <c r="G39" s="10"/>
+      <c r="H39" s="10"/>
+      <c r="I39" s="11"/>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A40" s="12"/>
+      <c r="B40" s="14"/>
+      <c r="C40" s="10"/>
+      <c r="D40" s="10"/>
+      <c r="E40" s="10"/>
+      <c r="F40" s="8"/>
+      <c r="G40" s="10"/>
+      <c r="H40" s="10"/>
+      <c r="I40" s="11"/>
     </row>
   </sheetData>
-  <mergeCells count="18">
-    <mergeCell ref="H12:H20"/>
-    <mergeCell ref="I1:I11"/>
-    <mergeCell ref="I12:I20"/>
-    <mergeCell ref="G2:G10"/>
-    <mergeCell ref="H3:H10"/>
+  <mergeCells count="36">
+    <mergeCell ref="E21:E30"/>
+    <mergeCell ref="F21:F30"/>
+    <mergeCell ref="G21:G30"/>
+    <mergeCell ref="H21:H30"/>
+    <mergeCell ref="I21:I30"/>
+    <mergeCell ref="A2:A10"/>
+    <mergeCell ref="A21:A30"/>
+    <mergeCell ref="C21:C30"/>
+    <mergeCell ref="D21:D30"/>
+    <mergeCell ref="B21:B30"/>
     <mergeCell ref="A11:A20"/>
-    <mergeCell ref="B11:B20"/>
-    <mergeCell ref="C11:C20"/>
-    <mergeCell ref="D11:D20"/>
-    <mergeCell ref="E11:E20"/>
     <mergeCell ref="F11:F20"/>
     <mergeCell ref="G11:G20"/>
     <mergeCell ref="B5:B10"/>
@@ -867,7 +1233,24 @@
     <mergeCell ref="D2:D10"/>
     <mergeCell ref="E2:E10"/>
     <mergeCell ref="F2:F10"/>
-    <mergeCell ref="A2:A10"/>
+    <mergeCell ref="B11:B20"/>
+    <mergeCell ref="C11:C20"/>
+    <mergeCell ref="D11:D20"/>
+    <mergeCell ref="E11:E20"/>
+    <mergeCell ref="H12:H20"/>
+    <mergeCell ref="I1:I11"/>
+    <mergeCell ref="I12:I20"/>
+    <mergeCell ref="G2:G10"/>
+    <mergeCell ref="H3:H10"/>
+    <mergeCell ref="F31:F40"/>
+    <mergeCell ref="G31:G40"/>
+    <mergeCell ref="H31:H40"/>
+    <mergeCell ref="I31:I40"/>
+    <mergeCell ref="A31:A40"/>
+    <mergeCell ref="B31:B40"/>
+    <mergeCell ref="C31:C40"/>
+    <mergeCell ref="D31:D40"/>
+    <mergeCell ref="E31:E40"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>